<commit_message>
#53 Completed Deliverables and BOM generated
</commit_message>
<xml_diff>
--- a/Design Files/Powermodule-v11.0.0/Deliverables/BOM/Client_BOM_Powermodule-v9.0.0.xlsx
+++ b/Design Files/Powermodule-v11.0.0/Deliverables/BOM/Client_BOM_Powermodule-v9.0.0.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="359">
   <si>
     <t>#</t>
   </si>
@@ -149,7 +149,7 @@
     <t>470nF</t>
   </si>
   <si>
-    <t>C15, C16, C63, C64</t>
+    <t>C15, C16, C63, C64,C67</t>
   </si>
   <si>
     <t>CAP CER 22UF 10V X5R 0402, Surface Mount Ceramic Multilayer Capacitor 100pF 2% C0G 50V 0201 Paper T/R</t>
@@ -398,6 +398,21 @@
     <t>Amphenol</t>
   </si>
   <si>
+    <t>LED_Pipe</t>
+  </si>
+  <si>
+    <t>J10</t>
+  </si>
+  <si>
+    <t>LED INDICATION, ROUND, CLEAR, DO</t>
+  </si>
+  <si>
+    <t>LPAV3-160-1000D-1-4</t>
+  </si>
+  <si>
+    <t>Bivar</t>
+  </si>
+  <si>
     <t>Battery Connector</t>
   </si>
   <si>
@@ -596,7 +611,7 @@
     <t>560R</t>
   </si>
   <si>
-    <t>R2, R8, R11, R12, R13, R30, R34, R59, R71, R72, R73</t>
+    <t>R2, R8, R11, R12, R13,R29, R30, R34, R59, R71, R72, R73</t>
   </si>
   <si>
     <t>RES 100K OHM 1% 1/16W 0402</t>
@@ -635,7 +650,7 @@
     <t>200R</t>
   </si>
   <si>
-    <t>R5, R6, R21, R25, R26, R37, R53, R54, R61, R65, R66, R69, R70</t>
+    <t>R5, R6, R21, R25, R26, R35,R37, R53, R54, R61, R65, R66, R69, R70</t>
   </si>
   <si>
     <t>RES 10K OHM 1% 1/16W 0402</t>
@@ -647,6 +662,9 @@
     <t>10K</t>
   </si>
   <si>
+    <t>R35 is DNP</t>
+  </si>
+  <si>
     <t>Resistors</t>
   </si>
   <si>
@@ -677,7 +695,7 @@
     <t>R10, R43, R60</t>
   </si>
   <si>
-    <t>R14, R15, R29, R57</t>
+    <t>R14, R15, R57</t>
   </si>
   <si>
     <t>RES 4.7K OHM 1% 1/16W 0402</t>
@@ -1098,7 +1116,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1190,14 +1208,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <strike/>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
@@ -1206,6 +1216,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1770,137 +1781,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1938,6 +1949,15 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1957,9 +1977,6 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1969,10 +1986,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2300,7 +2317,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="2" customWidth="1"/>
@@ -2327,9 +2344,9 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
     </row>
     <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="3"/>
@@ -2552,7 +2569,7 @@
         <v>43</v>
       </c>
       <c r="J8" s="12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" s="12"/>
     </row>
@@ -3036,7 +3053,7 @@
       </c>
       <c r="K23" s="10"/>
     </row>
-    <row r="24" ht="15.75" spans="1:11">
+    <row r="24" spans="1:11">
       <c r="A24" s="3"/>
       <c r="B24" s="8">
         <f t="shared" si="0"/>
@@ -3068,399 +3085,396 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" ht="36.75" spans="1:11">
+    <row r="25" spans="1:11">
       <c r="A25" s="3"/>
       <c r="B25" s="8">
-        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="17" t="s">
         <v>125</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="I25" s="11" t="s">
+      <c r="I25" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="J25" s="10">
+      <c r="J25" s="16">
         <v>1</v>
       </c>
-      <c r="K25" s="10"/>
-    </row>
-    <row r="26" ht="15.75" spans="1:11">
+      <c r="K25" s="16"/>
+    </row>
+    <row r="26" ht="36.75" spans="1:11">
       <c r="A26" s="3"/>
       <c r="B26" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B26)-ROW($B$2)</f>
         <v>24</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="D26" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="11" t="s">
         <v>130</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="H26" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="I26" s="13" t="s">
+      <c r="H26" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="I26" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J26" s="10">
         <v>1</v>
       </c>
-      <c r="K26" s="12"/>
-    </row>
-    <row r="27" ht="24.75" spans="1:11">
+      <c r="K26" s="10"/>
+    </row>
+    <row r="27" ht="15.75" spans="1:11">
       <c r="A27" s="3"/>
       <c r="B27" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B27)-ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D27" s="10" t="s">
+      <c r="C27" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="D27" s="12" t="s">
         <v>134</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>135</v>
       </c>
       <c r="F27" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="H27" s="10" t="s">
+      <c r="G27" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="I27" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="J27" s="10">
+      <c r="H27" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J27" s="12">
         <v>1</v>
       </c>
-      <c r="K27" s="10"/>
-    </row>
-    <row r="28" ht="15.75" spans="1:11">
+      <c r="K27" s="12"/>
+    </row>
+    <row r="28" ht="24.75" spans="1:11">
       <c r="A28" s="3"/>
       <c r="B28" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B28)-ROW($B$2)</f>
         <v>26</v>
       </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="12" t="s">
+      <c r="C28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="11" t="s">
         <v>139</v>
       </c>
       <c r="F28" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="H28" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="I28" s="13" t="s">
+      <c r="H28" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="J28" s="12">
+      <c r="I28" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="J28" s="10">
         <v>1</v>
       </c>
-      <c r="K28" s="12"/>
-    </row>
-    <row r="29" ht="24.75" spans="1:11">
+      <c r="K28" s="10"/>
+    </row>
+    <row r="29" ht="15.75" spans="1:11">
       <c r="A29" s="3"/>
       <c r="B29" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B29)-ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="D29" s="10" t="s">
+      <c r="C29" s="14"/>
+      <c r="D29" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="E29" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G29" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="H29" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="H29" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="I29" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="J29" s="10">
-        <v>3</v>
-      </c>
-      <c r="K29" s="10"/>
+      <c r="J29" s="12">
+        <v>1</v>
+      </c>
+      <c r="K29" s="12"/>
     </row>
     <row r="30" ht="24.75" spans="1:11">
       <c r="A30" s="3"/>
       <c r="B30" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B30)-ROW($B$2)</f>
         <v>28</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="D30" s="15" t="s">
+      <c r="C30" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E30" s="16" t="s">
+      <c r="E30" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="F30" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="G30" s="16" t="s">
+      <c r="F30" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="G30" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J30" s="10">
+        <v>3</v>
+      </c>
+      <c r="K30" s="10"/>
+    </row>
+    <row r="31" ht="24.75" spans="1:11">
+      <c r="A31" s="3"/>
+      <c r="B31" s="8">
+        <f>ROW(B31)-ROW($B$2)</f>
+        <v>29</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="I30" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="J30" s="15">
+      <c r="D31" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="H31" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="I31" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="J31" s="18">
         <v>1</v>
       </c>
-      <c r="K30" s="26" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="31" s="1" customFormat="1" ht="48.75" spans="1:18">
-      <c r="A31" s="17"/>
-      <c r="B31" s="18">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="F31" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="G31" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="H31" s="22" t="s">
+      <c r="K31" s="28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" s="1" customFormat="1" ht="48.75" spans="1:18">
+      <c r="A32" s="20"/>
+      <c r="B32" s="21">
+        <f>ROW(B32)-ROW($B$2)</f>
+        <v>30</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="H32" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I31" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="J31" s="20">
+      <c r="I32" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="J32" s="23">
         <v>33</v>
       </c>
-      <c r="K31" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="M31"/>
-      <c r="N31"/>
-      <c r="O31"/>
-      <c r="P31"/>
-      <c r="Q31"/>
-      <c r="R31"/>
-    </row>
-    <row r="32" ht="36.75" spans="1:11">
-      <c r="A32" s="3"/>
-      <c r="B32" s="8">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="C32" s="14" t="s">
+      <c r="K32" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="D32" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="F32" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="G32" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="H32" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J32" s="12">
-        <v>1</v>
-      </c>
-      <c r="K32" s="12"/>
+      <c r="M32"/>
+      <c r="N32"/>
+      <c r="O32"/>
+      <c r="P32"/>
+      <c r="Q32"/>
+      <c r="R32"/>
     </row>
     <row r="33" ht="36.75" spans="1:11">
       <c r="A33" s="3"/>
       <c r="B33" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B33)-ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D33" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="E33" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="E33" s="11" t="s">
+      <c r="F33" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="H33" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="I33" s="11" t="s">
+      <c r="I33" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J33" s="10">
-        <v>2</v>
-      </c>
-      <c r="K33" s="10"/>
-    </row>
-    <row r="34" ht="15.75" spans="1:11">
+      <c r="J33" s="12">
+        <v>1</v>
+      </c>
+      <c r="K33" s="12"/>
+    </row>
+    <row r="34" ht="36.75" spans="1:11">
       <c r="A34" s="3"/>
       <c r="B34" s="8">
-        <f t="shared" si="0"/>
+        <f>ROW(B34)-ROW($B$2)</f>
         <v>32</v>
       </c>
-      <c r="C34" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="D34" s="12" t="s">
+      <c r="C34" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="D34" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="F34" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="G34" s="13" t="s">
+      <c r="E34" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="12" t="s">
+      <c r="F34" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="I34" s="13" t="s">
+      <c r="H34" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="I34" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J34" s="12">
-        <v>1</v>
-      </c>
-      <c r="K34" s="12"/>
+      <c r="J34" s="10">
+        <v>2</v>
+      </c>
+      <c r="K34" s="10"/>
     </row>
     <row r="35" ht="15.75" spans="1:11">
       <c r="A35" s="3"/>
       <c r="B35" s="8">
-        <f t="shared" ref="B35:B66" si="1">ROW(B35)-ROW($B$2)</f>
+        <f>ROW(B35)-ROW($B$2)</f>
         <v>33</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="D35" s="10" t="s">
+      <c r="C35" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="E35" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="F35" s="10" t="s">
+      <c r="F35" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="G35" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="H35" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="H35" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="I35" s="11" t="s">
+      <c r="I35" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J35" s="10">
+      <c r="J35" s="12">
         <v>1</v>
       </c>
-      <c r="K35" s="10"/>
+      <c r="K35" s="12"/>
     </row>
     <row r="36" ht="15.75" spans="1:11">
       <c r="A36" s="3"/>
       <c r="B36" s="8">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B36:B67" si="1">ROW(B36)-ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="C36" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D36" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="D36" s="15" t="s">
+      <c r="E36" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="E36" s="16" t="s">
+      <c r="F36" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="F36" s="15" t="s">
+      <c r="G36" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="G36" s="16" t="s">
+      <c r="H36" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="H36" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="I36" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="J36" s="15">
+      <c r="I36" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J36" s="10">
         <v>1</v>
       </c>
-      <c r="K36" s="26" t="s">
-        <v>152</v>
-      </c>
+      <c r="K36" s="10"/>
     </row>
     <row r="37" ht="15.75" spans="1:11">
       <c r="A37" s="3"/>
@@ -3468,95 +3482,97 @@
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="E37" s="11" t="s">
+      <c r="E37" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="G37" s="11" t="s">
+      <c r="G37" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="H37" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I37" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="J37" s="10">
+      <c r="H37" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="I37" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="J37" s="18">
         <v>1</v>
       </c>
-      <c r="K37" s="10"/>
-    </row>
-    <row r="38" ht="24.75" spans="1:11">
+      <c r="K37" s="28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" spans="1:11">
       <c r="A38" s="3"/>
       <c r="B38" s="8">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="C38" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D38" s="12" t="s">
+      <c r="C38" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="F38" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G38" s="13" t="s">
+      <c r="F38" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="H38" s="12" t="s">
+      <c r="G38" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="H38" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I38" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="J38" s="12">
-        <v>11</v>
-      </c>
-      <c r="K38" s="12"/>
-    </row>
-    <row r="39" ht="15.75" spans="1:11">
+      <c r="I38" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="J38" s="10">
+        <v>1</v>
+      </c>
+      <c r="K38" s="10"/>
+    </row>
+    <row r="39" ht="24.75" spans="1:11">
       <c r="A39" s="3"/>
       <c r="B39" s="8">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="E39" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D39" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="F39" s="10" t="s">
+      <c r="E39" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="G39" s="11" t="s">
+      <c r="F39" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G39" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H39" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I39" s="11" t="s">
+      <c r="I39" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="J39" s="10">
-        <v>1</v>
-      </c>
-      <c r="K39" s="10"/>
+      <c r="J39" s="12">
+        <v>12</v>
+      </c>
+      <c r="K39" s="12"/>
     </row>
     <row r="40" ht="15.75" spans="1:11">
       <c r="A40" s="3"/>
@@ -3565,95 +3581,95 @@
         <v>38</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D40" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="E40" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="F40" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G40" s="13" t="s">
+      <c r="F40" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="H40" s="12" t="s">
+      <c r="G40" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="H40" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I40" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="J40" s="12">
-        <v>3</v>
-      </c>
-      <c r="K40" s="12"/>
-    </row>
-    <row r="41" ht="24.75" spans="1:11">
+      <c r="I40" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="J40" s="10">
+        <v>1</v>
+      </c>
+      <c r="K40" s="10"/>
+    </row>
+    <row r="41" ht="15.75" spans="1:11">
       <c r="A41" s="3"/>
       <c r="B41" s="8">
         <f t="shared" si="1"/>
         <v>39</v>
       </c>
-      <c r="C41" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="E41" s="11" t="s">
+      <c r="C41" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="F41" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="G41" s="11" t="s">
+      <c r="E41" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="F41" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G41" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I41" s="11" t="s">
-        <v>205</v>
-      </c>
-      <c r="J41" s="10">
-        <v>13</v>
-      </c>
-      <c r="K41" s="27"/>
-    </row>
-    <row r="42" ht="15.75" spans="1:11">
+      <c r="I41" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="J41" s="12">
+        <v>3</v>
+      </c>
+      <c r="K41" s="12"/>
+    </row>
+    <row r="42" ht="24.75" spans="1:11">
       <c r="A42" s="3"/>
       <c r="B42" s="8">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="C42" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="D42" s="15" t="s">
+      <c r="C42" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D42" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="E42" s="16" t="s">
+      <c r="E42" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="F42" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="G42" s="16" t="s">
+      <c r="F42" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="G42" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="H42" s="15" t="s">
+      <c r="H42" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I42" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="J42" s="15">
-        <v>1</v>
-      </c>
-      <c r="K42" s="26" t="s">
-        <v>152</v>
+      <c r="I42" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="J42" s="10">
+        <v>14</v>
+      </c>
+      <c r="K42" s="29" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="43" ht="15.75" spans="1:11">
@@ -3662,29 +3678,33 @@
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="F43" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="G43" s="11" t="s">
+      <c r="C43" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="D43" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="I43" s="11" t="s">
+      <c r="E43" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="J43" s="10">
-        <v>6</v>
-      </c>
-      <c r="K43" s="10"/>
+      <c r="F43" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="G43" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="H43" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I43" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="J43" s="18">
+        <v>1</v>
+      </c>
+      <c r="K43" s="28" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="44" ht="15.75" spans="1:11">
       <c r="A44" s="3"/>
@@ -3692,33 +3712,29 @@
         <f t="shared" si="1"/>
         <v>42</v>
       </c>
-      <c r="C44" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D44" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="E44" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="F44" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="G44" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="H44" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="I44" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="J44" s="15">
-        <v>3</v>
-      </c>
-      <c r="K44" s="26" t="s">
-        <v>152</v>
-      </c>
+      <c r="C44" s="9"/>
+      <c r="D44" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="G44" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="J44" s="10">
+        <v>6</v>
+      </c>
+      <c r="K44" s="10"/>
     </row>
     <row r="45" ht="15.75" spans="1:11">
       <c r="A45" s="3"/>
@@ -3726,97 +3742,97 @@
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="F45" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="G45" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H45" s="10" t="s">
+      <c r="C45" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F45" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="G45" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="H45" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="I45" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="J45" s="10">
-        <v>4</v>
-      </c>
-      <c r="K45" s="10"/>
-    </row>
-    <row r="46" ht="36.75" spans="1:11">
+      <c r="I45" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="J45" s="18">
+        <v>3</v>
+      </c>
+      <c r="K45" s="28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" spans="1:11">
       <c r="A46" s="3"/>
       <c r="B46" s="8">
         <f t="shared" si="1"/>
         <v>44</v>
       </c>
-      <c r="C46" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D46" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G46" s="13" t="s">
+      <c r="C46" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D46" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="H46" s="12" t="s">
+      <c r="E46" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="I46" s="13" t="s">
+      <c r="F46" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="G46" s="11" t="s">
         <v>224</v>
       </c>
-      <c r="J46" s="12">
-        <v>2</v>
-      </c>
-      <c r="K46" s="12"/>
-    </row>
-    <row r="47" ht="15.75" spans="1:11">
+      <c r="H46" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I46" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="J46" s="10">
+        <v>3</v>
+      </c>
+      <c r="K46" s="10"/>
+    </row>
+    <row r="47" ht="36.75" spans="1:11">
       <c r="A47" s="3"/>
       <c r="B47" s="8">
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D47" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="E47" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="F47" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="G47" s="24" t="s">
-        <v>218</v>
-      </c>
-      <c r="H47" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="J47" s="23">
+      <c r="C47" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G47" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="I47" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="J47" s="12">
         <v>2</v>
       </c>
-      <c r="K47" s="26" t="s">
-        <v>152</v>
-      </c>
+      <c r="K47" s="12"/>
     </row>
     <row r="48" ht="15.75" spans="1:11">
       <c r="A48" s="3"/>
@@ -3824,32 +3840,32 @@
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="C48" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D48" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="E48" s="16" t="s">
-        <v>227</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="G48" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="H48" s="15" t="s">
+      <c r="C48" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D48" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="E48" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="F48" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="G48" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="H48" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I48" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="J48" s="15">
+      <c r="I48" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="J48" s="25">
         <v>2</v>
       </c>
-      <c r="K48" s="26" t="s">
-        <v>152</v>
+      <c r="K48" s="28" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="49" ht="15.75" spans="1:11">
@@ -3858,31 +3874,33 @@
         <f t="shared" si="1"/>
         <v>47</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="F49" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="G49" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="H49" s="10" t="s">
+      <c r="C49" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="F49" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="G49" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="H49" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="I49" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="J49" s="10">
-        <v>1</v>
-      </c>
-      <c r="K49" s="10"/>
+      <c r="I49" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="J49" s="18">
+        <v>2</v>
+      </c>
+      <c r="K49" s="28" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="50" ht="15.75" spans="1:11">
       <c r="A50" s="3"/>
@@ -3890,33 +3908,31 @@
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="C50" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D50" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="E50" s="16" t="s">
-        <v>211</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="G50" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="H50" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="I50" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="J50" s="15">
+      <c r="C50" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="G50" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I50" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="J50" s="10">
         <v>1</v>
       </c>
-      <c r="K50" s="26" t="s">
-        <v>152</v>
-      </c>
+      <c r="K50" s="10"/>
     </row>
     <row r="51" ht="15.75" spans="1:11">
       <c r="A51" s="3"/>
@@ -3924,31 +3940,33 @@
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="C51" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="F51" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="G51" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I51" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="J51" s="10">
+      <c r="C51" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="F51" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="G51" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="H51" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="I51" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="J51" s="18">
         <v>1</v>
       </c>
-      <c r="K51" s="10"/>
+      <c r="K51" s="28" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="52" ht="15.75" spans="1:11">
       <c r="A52" s="3"/>
@@ -3956,31 +3974,31 @@
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="C52" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D52" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="F52" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G52" s="13" t="s">
+      <c r="C52" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D52" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="H52" s="12" t="s">
+      <c r="E52" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="G52" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="H52" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I52" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="J52" s="12">
-        <v>4</v>
-      </c>
-      <c r="K52" s="12"/>
+      <c r="I52" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="J52" s="10">
+        <v>1</v>
+      </c>
+      <c r="K52" s="10"/>
     </row>
     <row r="53" ht="15.75" spans="1:11">
       <c r="A53" s="3"/>
@@ -3988,31 +4006,31 @@
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
-      <c r="C53" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="E53" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="F53" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="G53" s="11" t="s">
+      <c r="C53" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D53" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="H53" s="10" t="s">
+      <c r="E53" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G53" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="H53" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I53" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="J53" s="10">
-        <v>1</v>
-      </c>
-      <c r="K53" s="10"/>
+      <c r="I53" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="J53" s="12">
+        <v>4</v>
+      </c>
+      <c r="K53" s="12"/>
     </row>
     <row r="54" ht="15.75" spans="1:11">
       <c r="A54" s="3"/>
@@ -4020,31 +4038,31 @@
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
-      <c r="C54" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D54" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="E54" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="F54" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G54" s="13" t="s">
+      <c r="C54" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D54" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="H54" s="12" t="s">
+      <c r="E54" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="G54" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="H54" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I54" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="J54" s="12">
+      <c r="I54" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="J54" s="10">
         <v>1</v>
       </c>
-      <c r="K54" s="12"/>
+      <c r="K54" s="10"/>
     </row>
     <row r="55" ht="15.75" spans="1:11">
       <c r="A55" s="3"/>
@@ -4052,31 +4070,31 @@
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
-      <c r="C55" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="E55" s="11" t="s">
-        <v>251</v>
-      </c>
-      <c r="F55" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="G55" s="11" t="s">
+      <c r="C55" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D55" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="H55" s="10" t="s">
+      <c r="E55" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G55" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="H55" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I55" s="11" t="s">
-        <v>253</v>
-      </c>
-      <c r="J55" s="10">
+      <c r="I55" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="J55" s="12">
         <v>1</v>
       </c>
-      <c r="K55" s="10"/>
+      <c r="K55" s="12"/>
     </row>
     <row r="56" ht="15.75" spans="1:11">
       <c r="A56" s="3"/>
@@ -4084,31 +4102,31 @@
         <f t="shared" si="1"/>
         <v>54</v>
       </c>
-      <c r="C56" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="D56" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="E56" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="F56" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G56" s="13" t="s">
+      <c r="C56" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D56" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="H56" s="12" t="s">
+      <c r="E56" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="G56" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="H56" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I56" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="J56" s="12">
-        <v>3</v>
-      </c>
-      <c r="K56" s="12"/>
+      <c r="I56" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="J56" s="10">
+        <v>1</v>
+      </c>
+      <c r="K56" s="10"/>
     </row>
     <row r="57" ht="15.75" spans="1:11">
       <c r="A57" s="3"/>
@@ -4116,65 +4134,65 @@
         <f t="shared" si="1"/>
         <v>55</v>
       </c>
-      <c r="C57" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="D57" s="23" t="s">
-        <v>258</v>
-      </c>
-      <c r="E57" s="24" t="s">
-        <v>255</v>
-      </c>
-      <c r="F57" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="G57" s="24" t="s">
-        <v>256</v>
-      </c>
-      <c r="H57" s="23" t="s">
+      <c r="C57" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G57" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="H57" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="I57" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="J57" s="23">
-        <v>1</v>
-      </c>
-      <c r="K57" s="26" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="58" ht="24.75" spans="1:11">
+      <c r="I57" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="J57" s="12">
+        <v>3</v>
+      </c>
+      <c r="K57" s="12"/>
+    </row>
+    <row r="58" ht="15.75" spans="1:11">
       <c r="A58" s="3"/>
       <c r="B58" s="8">
         <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="C58" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D58" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="E58" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="F58" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="G58" s="13" t="s">
+      <c r="C58" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="D58" s="25" t="s">
+        <v>264</v>
+      </c>
+      <c r="E58" s="26" t="s">
         <v>261</v>
       </c>
-      <c r="H58" s="12" t="s">
+      <c r="F58" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="G58" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="I58" s="13" t="s">
-        <v>263</v>
-      </c>
-      <c r="J58" s="12">
+      <c r="H58" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="I58" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="J58" s="25">
         <v>1</v>
       </c>
-      <c r="K58" s="12"/>
+      <c r="K58" s="28" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="59" ht="24.75" spans="1:11">
       <c r="A59" s="3"/>
@@ -4182,161 +4200,161 @@
         <f t="shared" si="1"/>
         <v>57</v>
       </c>
-      <c r="C59" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="E59" s="11" t="s">
+      <c r="C59" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D59" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="F59" s="10" t="s">
+      <c r="E59" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="G59" s="11" t="s">
+      <c r="F59" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="G59" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="H59" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="I59" s="11" t="s">
+      <c r="H59" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="J59" s="10">
+      <c r="I59" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="J59" s="12">
         <v>1</v>
       </c>
-      <c r="K59" s="10"/>
-    </row>
-    <row r="60" ht="36.75" spans="1:11">
+      <c r="K59" s="12"/>
+    </row>
+    <row r="60" ht="24.75" spans="1:11">
       <c r="A60" s="3"/>
       <c r="B60" s="8">
         <f t="shared" si="1"/>
         <v>58</v>
       </c>
-      <c r="C60" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="D60" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E60" s="13" t="s">
+      <c r="C60" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D60" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="F60" s="12" t="s">
-        <v>266</v>
-      </c>
-      <c r="G60" s="13" t="s">
+      <c r="E60" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="H60" s="12" t="s">
-        <v>262</v>
-      </c>
-      <c r="I60" s="13" t="s">
+      <c r="F60" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="J60" s="12">
+      <c r="G60" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="H60" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>274</v>
+      </c>
+      <c r="J60" s="10">
         <v>1</v>
       </c>
-      <c r="K60" s="12"/>
-    </row>
-    <row r="61" ht="15.75" spans="1:11">
+      <c r="K60" s="10"/>
+    </row>
+    <row r="61" ht="36.75" spans="1:11">
       <c r="A61" s="3"/>
       <c r="B61" s="8">
         <f t="shared" si="1"/>
         <v>59</v>
       </c>
-      <c r="C61" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="D61" s="23" t="s">
-        <v>274</v>
-      </c>
-      <c r="E61" s="24" t="s">
+      <c r="C61" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D61" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="F61" s="23" t="s">
+      <c r="E61" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="G61" s="24" t="s">
-        <v>276</v>
-      </c>
-      <c r="H61" s="23" t="s">
+      <c r="F61" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="G61" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="I61" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="J61" s="23">
+      <c r="H61" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="I61" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="J61" s="12">
         <v>1</v>
       </c>
-      <c r="K61" s="26" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="62" ht="36.75" spans="1:11">
+      <c r="K61" s="12"/>
+    </row>
+    <row r="62" ht="15.75" spans="1:11">
       <c r="A62" s="3"/>
       <c r="B62" s="8">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="D62" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="E62" s="13" t="s">
         <v>279</v>
       </c>
-      <c r="F62" s="12" t="s">
+      <c r="D62" s="25" t="s">
         <v>280</v>
       </c>
-      <c r="G62" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="H62" s="12" t="s">
+      <c r="E62" s="26" t="s">
         <v>281</v>
       </c>
-      <c r="I62" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J62" s="12">
-        <v>2</v>
-      </c>
-      <c r="K62" s="12"/>
-    </row>
-    <row r="63" ht="15.75" spans="1:11">
+      <c r="F62" s="25" t="s">
+        <v>282</v>
+      </c>
+      <c r="G62" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="H62" s="25" t="s">
+        <v>283</v>
+      </c>
+      <c r="I62" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="J62" s="25">
+        <v>1</v>
+      </c>
+      <c r="K62" s="28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="63" ht="36.75" spans="1:11">
       <c r="A63" s="3"/>
       <c r="B63" s="8">
         <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="D63" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="E63" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="D63" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="F63" s="10" t="s">
+      <c r="E63" s="13" t="s">
         <v>285</v>
       </c>
-      <c r="G63" s="11" t="s">
+      <c r="F63" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="H63" s="10" t="s">
+      <c r="G63" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="H63" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="I63" s="11" t="s">
+      <c r="I63" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J63" s="10">
-        <v>1</v>
-      </c>
-      <c r="K63" s="10"/>
+      <c r="J63" s="12">
+        <v>2</v>
+      </c>
+      <c r="K63" s="12"/>
     </row>
     <row r="64" ht="15.75" spans="1:11">
       <c r="A64" s="3"/>
@@ -4344,189 +4362,189 @@
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="C64" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D64" s="12" t="s">
+      <c r="C64" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="E64" s="13" t="s">
+      <c r="D64" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="F64" s="12" t="s">
+      <c r="E64" s="11" t="s">
         <v>290</v>
       </c>
-      <c r="G64" s="13" t="s">
+      <c r="F64" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="H64" s="12" t="s">
-        <v>287</v>
-      </c>
-      <c r="I64" s="13" t="s">
+      <c r="G64" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="H64" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="I64" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J64" s="12">
+      <c r="J64" s="10">
         <v>1</v>
       </c>
-      <c r="K64" s="12"/>
-    </row>
-    <row r="65" ht="24.75" spans="1:11">
+      <c r="K64" s="10"/>
+    </row>
+    <row r="65" ht="15.75" spans="1:11">
       <c r="A65" s="3"/>
       <c r="B65" s="8">
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>292</v>
-      </c>
-      <c r="E65" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="F65" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="G65" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="H65" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="F65" s="10" t="s">
-        <v>294</v>
-      </c>
-      <c r="G65" s="11" t="s">
-        <v>295</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>296</v>
-      </c>
-      <c r="I65" s="11" t="s">
+      <c r="I65" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J65" s="10">
+      <c r="J65" s="12">
         <v>1</v>
       </c>
-      <c r="K65" s="10"/>
-    </row>
-    <row r="66" ht="15.75" spans="1:11">
+      <c r="K65" s="12"/>
+    </row>
+    <row r="66" ht="24.75" spans="1:11">
       <c r="A66" s="3"/>
       <c r="B66" s="8">
         <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D66" s="12" t="s">
-        <v>297</v>
-      </c>
-      <c r="E66" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="D66" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="F66" s="12" t="s">
+      <c r="E66" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="G66" s="13" t="s">
+      <c r="F66" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="H66" s="12" t="s">
+      <c r="G66" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="I66" s="13" t="s">
+      <c r="H66" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="I66" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J66" s="12">
+      <c r="J66" s="10">
         <v>1</v>
       </c>
-      <c r="K66" s="12"/>
-    </row>
-    <row r="67" ht="36.75" spans="1:11">
+      <c r="K66" s="10"/>
+    </row>
+    <row r="67" ht="15.75" spans="1:11">
       <c r="A67" s="3"/>
       <c r="B67" s="8">
-        <f t="shared" ref="B67:B78" si="2">ROW(B67)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>65</v>
       </c>
-      <c r="C67" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="D67" s="10" t="s">
+      <c r="C67" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D67" s="12" t="s">
         <v>303</v>
       </c>
-      <c r="E67" s="11" t="s">
+      <c r="E67" s="13" t="s">
         <v>304</v>
       </c>
-      <c r="F67" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="G67" s="11" t="s">
+      <c r="F67" s="12" t="s">
         <v>305</v>
       </c>
-      <c r="H67" s="10" t="s">
+      <c r="G67" s="13" t="s">
         <v>306</v>
       </c>
-      <c r="I67" s="11" t="s">
+      <c r="H67" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="I67" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J67" s="10">
-        <v>4</v>
-      </c>
-      <c r="K67" s="10"/>
-    </row>
-    <row r="68" ht="24.75" spans="1:11">
+      <c r="J67" s="12">
+        <v>1</v>
+      </c>
+      <c r="K67" s="12"/>
+    </row>
+    <row r="68" ht="36.75" spans="1:11">
       <c r="A68" s="3"/>
       <c r="B68" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="B68:B79" si="2">ROW(B68)-ROW($B$2)</f>
         <v>66</v>
       </c>
-      <c r="C68" s="14" t="s">
-        <v>307</v>
-      </c>
-      <c r="D68" s="12" t="s">
+      <c r="C68" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="E68" s="13" t="s">
+      <c r="D68" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="F68" s="12" t="s">
+      <c r="E68" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="F68" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="G68" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="H68" s="12"/>
-      <c r="I68" s="13" t="s">
+      <c r="G68" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="H68" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="I68" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J68" s="12">
-        <v>1</v>
-      </c>
-      <c r="K68" s="12"/>
-    </row>
-    <row r="69" ht="15.75" spans="1:11">
+      <c r="J68" s="10">
+        <v>4</v>
+      </c>
+      <c r="K68" s="10"/>
+    </row>
+    <row r="69" ht="24.75" spans="1:11">
       <c r="A69" s="3"/>
       <c r="B69" s="8">
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
-      <c r="C69" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="D69" s="10" t="s">
-        <v>311</v>
-      </c>
-      <c r="E69" s="11" t="s">
-        <v>312</v>
-      </c>
-      <c r="F69" s="10" t="s">
+      <c r="C69" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="G69" s="11" t="s">
+      <c r="D69" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="H69" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="I69" s="11" t="s">
+      <c r="E69" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="F69" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G69" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="H69" s="12"/>
+      <c r="I69" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J69" s="10">
+      <c r="J69" s="12">
         <v>1</v>
       </c>
-      <c r="K69" s="10"/>
+      <c r="K69" s="12"/>
     </row>
     <row r="70" ht="15.75" spans="1:11">
       <c r="A70" s="3"/>
@@ -4534,31 +4552,31 @@
         <f t="shared" si="2"/>
         <v>68</v>
       </c>
-      <c r="C70" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D70" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="E70" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="F70" s="12" t="s">
+      <c r="C70" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D70" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="G70" s="13" t="s">
+      <c r="E70" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="H70" s="12" t="s">
-        <v>287</v>
+      <c r="F70" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="H70" s="10" t="s">
+        <v>293</v>
       </c>
       <c r="I70" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J70" s="12">
+      <c r="J70" s="10">
         <v>1</v>
       </c>
-      <c r="K70" s="12"/>
+      <c r="K70" s="10"/>
     </row>
     <row r="71" ht="15.75" spans="1:11">
       <c r="A71" s="3"/>
@@ -4566,31 +4584,31 @@
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
-      <c r="C71" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>319</v>
-      </c>
-      <c r="E71" s="11" t="s">
-        <v>320</v>
-      </c>
-      <c r="F71" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="G71" s="11" t="s">
+      <c r="C71" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D71" s="12" t="s">
         <v>321</v>
       </c>
-      <c r="H71" s="10" t="s">
-        <v>287</v>
+      <c r="E71" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="F71" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="G71" s="13" t="s">
+        <v>324</v>
+      </c>
+      <c r="H71" s="12" t="s">
+        <v>293</v>
       </c>
       <c r="I71" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J71" s="10">
+      <c r="J71" s="12">
         <v>1</v>
       </c>
-      <c r="K71" s="10"/>
+      <c r="K71" s="12"/>
     </row>
     <row r="72" ht="15.75" spans="1:11">
       <c r="A72" s="3"/>
@@ -4598,95 +4616,95 @@
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
-      <c r="C72" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D72" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="E72" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="F72" s="12" t="s">
-        <v>324</v>
-      </c>
-      <c r="G72" s="13" t="s">
+      <c r="C72" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D72" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="H72" s="12" t="s">
-        <v>287</v>
+      <c r="E72" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="F72" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="G72" s="11" t="s">
+        <v>327</v>
+      </c>
+      <c r="H72" s="10" t="s">
+        <v>293</v>
       </c>
       <c r="I72" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J72" s="12">
+      <c r="J72" s="10">
         <v>1</v>
       </c>
-      <c r="K72" s="12"/>
-    </row>
-    <row r="73" ht="24.75" spans="1:11">
+      <c r="K72" s="10"/>
+    </row>
+    <row r="73" ht="15.75" spans="1:11">
       <c r="A73" s="3"/>
       <c r="B73" s="8">
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
-      <c r="C73" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>326</v>
-      </c>
-      <c r="E73" s="11" t="s">
-        <v>327</v>
-      </c>
-      <c r="F73" s="10" t="s">
+      <c r="C73" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D73" s="12" t="s">
         <v>328</v>
       </c>
-      <c r="G73" s="11" t="s">
-        <v>328</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>287</v>
+      <c r="E73" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="F73" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="G73" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="H73" s="12" t="s">
+        <v>293</v>
       </c>
       <c r="I73" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J73" s="10">
+      <c r="J73" s="12">
         <v>1</v>
       </c>
-      <c r="K73" s="10"/>
-    </row>
-    <row r="74" ht="15.75" spans="1:11">
+      <c r="K73" s="12"/>
+    </row>
+    <row r="74" ht="24.75" spans="1:11">
       <c r="A74" s="3"/>
       <c r="B74" s="8">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="C74" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D74" s="12" t="s">
-        <v>329</v>
-      </c>
-      <c r="E74" s="13" t="s">
-        <v>330</v>
-      </c>
-      <c r="F74" s="12" t="s">
-        <v>331</v>
-      </c>
-      <c r="G74" s="13" t="s">
+      <c r="C74" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D74" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="H74" s="12" t="s">
-        <v>287</v>
+      <c r="E74" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="F74" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="G74" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="H74" s="10" t="s">
+        <v>293</v>
       </c>
       <c r="I74" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J74" s="12">
+      <c r="J74" s="10">
         <v>1</v>
       </c>
-      <c r="K74" s="12"/>
+      <c r="K74" s="10"/>
     </row>
     <row r="75" ht="15.75" spans="1:11">
       <c r="A75" s="3"/>
@@ -4694,127 +4712,159 @@
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="C75" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="D75" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="E75" s="11" t="s">
-        <v>334</v>
-      </c>
-      <c r="F75" s="10" t="s">
+      <c r="C75" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D75" s="12" t="s">
         <v>335</v>
       </c>
-      <c r="G75" s="11" t="s">
+      <c r="E75" s="13" t="s">
         <v>336</v>
       </c>
-      <c r="H75" s="10" t="s">
+      <c r="F75" s="12" t="s">
         <v>337</v>
+      </c>
+      <c r="G75" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="H75" s="12" t="s">
+        <v>293</v>
       </c>
       <c r="I75" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J75" s="10">
+      <c r="J75" s="12">
         <v>1</v>
       </c>
-      <c r="K75" s="10"/>
-    </row>
-    <row r="76" ht="36.75" spans="1:11">
+      <c r="K75" s="12"/>
+    </row>
+    <row r="76" ht="15.75" spans="1:11">
       <c r="A76" s="3"/>
       <c r="B76" s="8">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="C76" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="D76" s="12" t="s">
+      <c r="C76" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D76" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="E76" s="13" t="s">
+      <c r="E76" s="11" t="s">
         <v>340</v>
       </c>
-      <c r="F76" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G76" s="13" t="s">
+      <c r="F76" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="H76" s="12" t="s">
+      <c r="G76" s="11" t="s">
         <v>342</v>
       </c>
-      <c r="I76" s="13" t="s">
+      <c r="H76" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="J76" s="12">
+      <c r="I76" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J76" s="10">
         <v>1</v>
       </c>
-      <c r="K76" s="12"/>
-    </row>
-    <row r="77" ht="24.75" spans="1:11">
+      <c r="K76" s="10"/>
+    </row>
+    <row r="77" ht="36.75" spans="1:11">
       <c r="A77" s="3"/>
       <c r="B77" s="8">
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="C77" s="9" t="s">
-        <v>338</v>
-      </c>
-      <c r="D77" s="10" t="s">
+      <c r="C77" s="14" t="s">
         <v>344</v>
       </c>
-      <c r="E77" s="11" t="s">
+      <c r="D77" s="12" t="s">
         <v>345</v>
       </c>
-      <c r="F77" s="10" t="s">
+      <c r="E77" s="13" t="s">
         <v>346</v>
       </c>
-      <c r="G77" s="11" t="s">
+      <c r="F77" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G77" s="13" t="s">
         <v>347</v>
       </c>
-      <c r="H77" s="10" t="s">
+      <c r="H77" s="12" t="s">
         <v>348</v>
       </c>
-      <c r="I77" s="11" t="s">
+      <c r="I77" s="13" t="s">
         <v>349</v>
       </c>
-      <c r="J77" s="10">
+      <c r="J77" s="12">
         <v>1</v>
       </c>
-      <c r="K77" s="10"/>
-    </row>
-    <row r="78" ht="15.75" spans="1:11">
+      <c r="K77" s="12"/>
+    </row>
+    <row r="78" ht="24.75" spans="1:11">
       <c r="A78" s="3"/>
       <c r="B78" s="8">
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
       <c r="C78" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="D78" s="10" t="s">
         <v>350</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="E78" s="11" t="s">
         <v>351</v>
       </c>
       <c r="F78" s="10" t="s">
-        <v>81</v>
+        <v>352</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>81</v>
+        <v>354</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>81</v>
+        <v>355</v>
       </c>
       <c r="J78" s="10">
         <v>1</v>
       </c>
       <c r="K78" s="10"/>
+    </row>
+    <row r="79" ht="15.75" spans="1:11">
+      <c r="A79" s="3"/>
+      <c r="B79" s="8">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="E79" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="F79" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G79" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="H79" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I79" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J79" s="10">
+        <v>1</v>
+      </c>
+      <c r="K79" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>